<commit_message>
Corrigindo rotas e atualização do app.py
</commit_message>
<xml_diff>
--- a/agenda.xlsx
+++ b/agenda.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D97"/>
+  <dimension ref="A1:D130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1695,44 +1695,44 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>esdra</t>
+          <t>darcy</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t xml:space="preserve">corte luzes sombracelha e barba </t>
+          <t xml:space="preserve">corte </t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>darcy</t>
+          <t>Lene</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t xml:space="preserve">corte </t>
+          <t xml:space="preserve">corte e barba </t>
         </is>
       </c>
     </row>
@@ -1815,46 +1815,46 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t xml:space="preserve">corte e barba </t>
+          <t xml:space="preserve">corte luzes sombracelha e barba </t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Lene</t>
+          <t>darcy</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t xml:space="preserve">corte luzes sombracelha e barba </t>
+          <t xml:space="preserve">corte </t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>darcy</t>
+          <t>Billy</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1871,12 +1871,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Billy</t>
+          <t>pastor Daniel</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1886,90 +1886,90 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t xml:space="preserve">corte </t>
+          <t xml:space="preserve">corte e barba </t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>pastor Daniel</t>
+          <t xml:space="preserve">brow </t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t xml:space="preserve">corte e barba </t>
+          <t>corte e barba e pigmentação</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">brow </t>
+          <t>gil</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>corte e barba e pigmentação</t>
+          <t xml:space="preserve">corte </t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>gil</t>
+          <t>luiz lorenço</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-27</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t xml:space="preserve">corte </t>
+          <t>corte e sombracelha</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>luiz lorenço</t>
+          <t>Antonio juma Lembi</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -1981,7 +1981,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Antonio juma Lembi</t>
+          <t>Ton mecanico</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1991,29 +1991,29 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>corte e sombracelha</t>
+          <t xml:space="preserve">corte e barba </t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Ton mecanico</t>
+          <t>dioclesio</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-20</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2025,51 +2025,51 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>dioclesio</t>
+          <t>lilica</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t xml:space="preserve">corte e barba </t>
+          <t xml:space="preserve">corte luzes </t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>lilica</t>
+          <t>shall</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t xml:space="preserve">corte luzes </t>
+          <t>Barba</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>shall</t>
+          <t>Lene</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2091,7 +2091,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Lene</t>
+          <t>shall</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2113,7 +2113,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>shall</t>
+          <t>Lene</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2135,7 +2135,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Lene</t>
+          <t>esdra</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2179,7 +2179,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>esdra</t>
+          <t>Lene</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2201,7 +2201,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Lene</t>
+          <t>esdra</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2211,7 +2211,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2223,7 +2223,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>esdra</t>
+          <t>Lene</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2233,12 +2233,12 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Barba</t>
+          <t>Corte</t>
         </is>
       </c>
     </row>
@@ -2255,12 +2255,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Corte</t>
+          <t>Corte e Barba</t>
         </is>
       </c>
     </row>
@@ -2277,12 +2277,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Corte e Barba</t>
+          <t>Barba</t>
         </is>
       </c>
     </row>
@@ -2299,12 +2299,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Barba</t>
+          <t>Corte + Sobrancelha</t>
         </is>
       </c>
     </row>
@@ -2321,12 +2321,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Corte + Sobrancelha</t>
+          <t>Barba</t>
         </is>
       </c>
     </row>
@@ -2343,12 +2343,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Barba</t>
+          <t>Corte e Barba</t>
         </is>
       </c>
     </row>
@@ -2365,19 +2365,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Corte e Barba</t>
+          <t>Barba</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Lene</t>
+          <t>esdra</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2387,34 +2387,34 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Barba</t>
+          <t>Corte</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>esdra</t>
+          <t xml:space="preserve">Paulo </t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Corte</t>
+          <t xml:space="preserve">corte e barba </t>
         </is>
       </c>
     </row>
@@ -2443,7 +2443,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paulo </t>
+          <t xml:space="preserve">paulo </t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2458,68 +2458,68 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t xml:space="preserve">corte e barba </t>
+          <t>Corte e Barba</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t xml:space="preserve">paulo </t>
+          <t>dj dennyboy</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2025-12-23</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Corte e Barba</t>
+          <t xml:space="preserve">corte e barba </t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>dj dennyboy</t>
+          <t>Lene</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t xml:space="preserve">corte e barba </t>
+          <t>Corte e Barba</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>josi</t>
+          <t xml:space="preserve">juninho </t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2536,17 +2536,743 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte e barba </t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Lene</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte e barba </t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Lene</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte e barba </t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Lene</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte e barba </t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Lene</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte e barba </t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Lene</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte e barba </t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Lene</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte e barba </t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Lene</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte e barba </t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Lene</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte e barba </t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Lene</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte e barba </t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Lene</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte e barba </t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Lene</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte e barba </t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Lene</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte e barba </t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>esdra</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte e barba </t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Lene</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Corte e Barba</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Lene</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte e barba </t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Lene</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte e barba </t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Lene</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte e barba </t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Lene</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte e barba </t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Lene</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte e barba </t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Lene</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte e barba </t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Billy</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>2025-12-27</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte </t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Lene</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
           <t>2025-12-30</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
-      <c r="D97" t="inlineStr">
-        <is>
-          <t>Corte e Barba</t>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Barba</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>marquito</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte e barba </t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">brow </t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte e barba </t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>kevin</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte </t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>claudinho</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte </t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ronaldo </t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">corte e barba </t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Lene</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Corte</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>shall</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Corte</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>liiiii</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Corte</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>liiiii</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Barba</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Lene</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Barba</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>esdra</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Barba</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Minha mensagem explicando o que eu mudei
</commit_message>
<xml_diff>
--- a/agenda.xlsx
+++ b/agenda.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D130"/>
+  <dimension ref="A1:D134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3276,6 +3276,94 @@
         </is>
       </c>
     </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>esdra</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Barba</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Lene</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Barba</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Lene</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Barba</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Lene</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Corte + Sobrancelha</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>